<commit_message>
Add Sold At timestamp + Source link columns to dashboard
</commit_message>
<xml_diff>
--- a/data/output/SurplusIQ_Leads_2026-05-06.xlsx
+++ b/data/output/SurplusIQ_Leads_2026-05-06.xlsx
@@ -613,7 +613,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: May 06, 2026 at 07:47 AM</t>
+          <t>Generated: May 06, 2026 at 01:36 PM</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated: May 06, 2026 at 07:47 AM | 29 leads</t>
+          <t>Generated: May 06, 2026 at 01:36 PM | 29 leads</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated: May 06, 2026 at 07:47 AM | 7 leads</t>
+          <t>Generated: May 06, 2026 at 01:36 PM | 7 leads</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated: May 06, 2026 at 07:47 AM | 15 leads</t>
+          <t>Generated: May 06, 2026 at 01:36 PM | 15 leads</t>
         </is>
       </c>
     </row>
@@ -4649,7 +4649,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated: May 06, 2026 at 07:47 AM | 14 leads</t>
+          <t>Generated: May 06, 2026 at 01:36 PM | 14 leads</t>
         </is>
       </c>
     </row>

</xml_diff>